<commit_message>
Wiersze z objaśnieniami w zestawieniu scalone na szerokość tabeli
Tekst objaśnień siedział w komórkach kolumny pierwszej, więc
w przeglądarce arkuszy łamał się w wąskim słupku obok pustych pól.
Osiem wierszy - tytuł, dwa wprowadzające i pięć legendy - jest teraz
scalonych od A do F.

Przy okazji wiersz wprowadzający powtarzał stare brzmienie, jakoby
prośba o finansowanie dotyczyła wierszy "tak"; mówi teraz to samo co
legenda i nota: kolumna wskazuje zakres pytania, nie prośbę o środki.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/attachments/zestawienie-zadania.xlsx
+++ b/attachments/zestawienie-zadania.xlsx
@@ -28,7 +28,7 @@
     <t xml:space="preserve">Załącznik do pisma do Ministerstwa Kultury i Dziedzictwa Narodowego. Kwoty netto, z arkusza budżetowego pierwszej edycji.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prośba o wskazanie drogi finansowania dotyczy wyłącznie wierszy oznaczonych "tak" w ostatniej kolumnie.</t>
+    <t xml:space="preserve">Ostatnia kolumna mówi, czy pozycja mieści się w zakresie pytania do Ministerstwa, a nie czy wnoszę o jej sfinansowanie. Objaśnienie pod tabelą.</t>
   </si>
   <si>
     <t xml:space="preserve">Działanie</t>
@@ -346,11 +346,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -394,11 +394,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -669,16 +669,31 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
@@ -1002,28 +1017,63 @@
       <c r="A24" s="14" t="s">
         <v>54</v>
       </c>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
         <v>55</v>
       </c>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
         <v>56</v>
       </c>
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
         <v>57</v>
       </c>
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
         <v>58</v>
       </c>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A29:F29"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Nagroda Uczniowska jako nagroda pieniężna: 10 000 zł brutto
Regulamin przyznawał ją bez kwoty, a w arkuszu nie było na nią pozycji,
więc laureat wskazany przez szkoły wychodziłby z gali z samym dyplomem -
także wtedy, gdy jego rozmowa nie weszła do dziesiątki. Nowy § 9 ust. 9
lit. a1 ustala 10 000 zł brutto i kumulację z werdyktem jury, nowy
wiersz w Budżecie Nagrody dokłada tę kwotę wraz z rezerwą. Budżet
Nagrody rośnie z 511 996,80 zł do 523 196,80 zł, suma wszystkich
wycenionych pozycji z 1 665 626,80 zł do 1 676 826,80 zł. Poprawiony
także opis nagród publiczności: 4 000 zł brutto w podziale 3 000 dla
rozmowy z największą liczbą głosów i 1 000 za uzasadnienie głosu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/attachments/zestawienie-zadania.xlsx
+++ b/attachments/zestawienie-zadania.xlsx
@@ -613,13 +613,13 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>511996.8</v>
+        <v>523196.8</v>
       </c>
       <c r="E6" s="25" t="n">
         <v>77156.8</v>
       </c>
       <c r="F6" s="25" t="n">
-        <v>434840</v>
+        <v>446040</v>
       </c>
       <c r="G6" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Nagrody publiczności po 12 000 zł w każdym plebiscycie
Podział jest wszędzie ten sam: 10 000 zł dla zgłoszenia z największą
liczbą głosów i 2 000 zł za najlepsze uzasadnienie oddanego głosu,
zamiast dotychczasowych 3 000 i 1 000. Głos publiczności waży tyle samo
w każdej z czterech dziedzin, niezależnie od wysokości puli jury.

Budżet Nagrody rośnie do 532 156,80 zł, plebiscytu na piosenkę do
262 600 zł, na plakat do 162 480 zł, na film do 264 800 zł. Zakres
objęty pytaniem do MKiDN rośnie z 660 952,00 zł do 684 952,00 zł, suma
wszystkich wycenionych pozycji z 1 676 826,80 zł do 1 709 786,80 zł.
Zwolnienie podatkowe z art. 21 ust. 1 pkt 68 nadal obejmuje nagrodę za
uzasadnienie, bo 2 000 zł nie przekracza progu.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/attachments/zestawienie-zadania.xlsx
+++ b/attachments/zestawienie-zadania.xlsx
@@ -613,13 +613,13 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>523196.8</v>
+        <v>532156.8</v>
       </c>
       <c r="E6" s="25" t="n">
         <v>77156.8</v>
       </c>
       <c r="F6" s="25" t="n">
-        <v>446040</v>
+        <v>455000</v>
       </c>
       <c r="G6" s="26" t="inlineStr">
         <is>
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>99600</v>
+        <v>107600</v>
       </c>
       <c r="E10" s="25" t="n">
         <v>28080</v>
       </c>
       <c r="F10" s="25" t="n">
-        <v>71520</v>
+        <v>79520</v>
       </c>
       <c r="G10" s="26" t="inlineStr">
         <is>
@@ -913,13 +913,13 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>149552</v>
+        <v>157552</v>
       </c>
       <c r="E14" s="25" t="n">
         <v>17248</v>
       </c>
       <c r="F14" s="25" t="n">
-        <v>132304</v>
+        <v>140304</v>
       </c>
       <c r="G14" s="26" t="inlineStr">
         <is>
@@ -1029,13 +1029,13 @@
         </is>
       </c>
       <c r="D17" s="25" t="n">
-        <v>256800</v>
+        <v>264800</v>
       </c>
       <c r="E17" s="25" t="n">
         <v>32032</v>
       </c>
       <c r="F17" s="25" t="n">
-        <v>224768</v>
+        <v>232768</v>
       </c>
       <c r="G17" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rezerwa Budżetu Nagrody liczona bez nagród, jak w pozostałych budżetach
Nagrody publiczności i Nagroda Uczniowska stały w kosztach twardych, a
rezerwa 12% naliczała się od nich - choć etykieta pozycji mówi "bez
nagród", a trzy pozostałe budżety tak właśnie liczą. Po wyłączeniu obu
pozycji z podstawy Budżet Nagrody spada z 532 156,80 zł do
529 516,80 zł, a suma wszystkich wycenionych pozycji do 1 707 146,80 zł.
Zakres objęty pytaniem do MKiDN bez zmian, bo plebiscyt na rozmowę do
niego nie należy.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/attachments/zestawienie-zadania.xlsx
+++ b/attachments/zestawienie-zadania.xlsx
@@ -613,13 +613,13 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>532156.8</v>
+        <v>529516.8</v>
       </c>
       <c r="E6" s="25" t="n">
         <v>77156.8</v>
       </c>
       <c r="F6" s="25" t="n">
-        <v>455000</v>
+        <v>452360</v>
       </c>
       <c r="G6" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Wydzielony Budżet Uruchomienia i rola Mecenasa Założycielskiego
Koszty wspólne całego przedsięwzięcia - powołanie fundacji i jej
obsługa, konsultacja prawna, domeny i hosting, narzędzia AI, znak
towarowy, przebudowa strony oraz trzy narzędzia obsługujące wszystkie
plebiscyty - wychodzą z Budżetu Antologii do osobnej zakładki i osobnej
roli. Obciążanie nimi jednego partnera znaczyło, że finansuje on
infrastrukturę dla pozostałych i sam ponosi ryzyko, że reszta ról nie
zostanie obsadzona.

Budżet Antologii spada z 344 422 zł do 180 362 zł netto, czyli
221 845,26 zł brutto; Budżet Uruchomienia to 164 060 zł netto. Suma
wszystkich pozycji bez zmian: 1 759 146,80 zł. Zestawienie zadania ma
nowy wiersz, a strona dla partnerów nowy kafel.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/attachments/zestawienie-zadania.xlsx
+++ b/attachments/zestawienie-zadania.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="46" customWidth="1" style="16" min="1" max="1"/>
@@ -673,12 +673,12 @@
     <row r="8" ht="23.25" customHeight="1" s="17">
       <c r="A8" s="26" t="inlineStr">
         <is>
-          <t>Antologia i Archiwum, w tym krótki nakład na galę</t>
+          <t>Antologia, Archiwum i podcast</t>
         </is>
       </c>
       <c r="B8" s="26" t="inlineStr">
         <is>
-          <t>e-book bezpłatny, audiobook, Archiwum, egzemplarze dla laureatów</t>
+          <t>e-book bezpłatny, audiobook, wydanie książkowe, Archiwum</t>
         </is>
       </c>
       <c r="C8" s="27" t="inlineStr">
@@ -687,10 +687,10 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>344422</v>
+        <v>180362</v>
       </c>
       <c r="E8" s="25" t="n">
-        <v>201812</v>
+        <v>37752</v>
       </c>
       <c r="F8" s="25" t="n">
         <v>142610</v>
@@ -709,31 +709,33 @@
     <row r="9" ht="23.25" customHeight="1" s="17">
       <c r="A9" s="26" t="inlineStr">
         <is>
-          <t>Pierwsza runda oceny: Akademia rozmów i akademia filmu</t>
+          <t>Uruchomienie: fundacja, znak towarowy, strona i narzędzia oceny</t>
         </is>
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>przesiew zgłoszeń, dwa odczyty rozmowy i dwa obejrzenia filmu na zgłoszenie</t>
+          <t>fundacja w KRS, regulamin po konsultacji prawnej, cztery narzędzia, przebudowana strona</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>2027-2028</t>
+          <t>2027</t>
         </is>
       </c>
       <c r="D9" s="25" t="n">
-        <v>160160</v>
+        <v>164060</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>59360</v>
-      </c>
-      <c r="F9" s="25" t="n">
-        <v>100800</v>
+        <v>164060</v>
+      </c>
+      <c r="F9" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G9" s="26" t="inlineStr">
         <is>
-          <t>sponsor akademii</t>
+          <t>mecenas założycielski</t>
         </is>
       </c>
       <c r="H9" s="27" t="inlineStr">
@@ -745,12 +747,12 @@
     <row r="10" ht="23.25" customHeight="1" s="17">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>Plebiscyt na piosenkę: nabór, ocena, nagrody, prowadzenie</t>
+          <t>Pierwsza runda oceny: Akademia rozmów i akademia filmu</t>
         </is>
       </c>
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>plebiscyt i jego laureaci</t>
+          <t>przesiew zgłoszeń, dwa odczyty rozmowy i dwa obejrzenia filmu na zgłoszenie</t>
         </is>
       </c>
       <c r="C10" s="27" t="inlineStr">
@@ -759,51 +761,49 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>107600</v>
+        <v>160160</v>
       </c>
       <c r="E10" s="25" t="n">
-        <v>28080</v>
+        <v>59360</v>
       </c>
       <c r="F10" s="25" t="n">
-        <v>79520</v>
+        <v>100800</v>
       </c>
       <c r="G10" s="26" t="inlineStr">
         <is>
-          <t>sponsor plebiscytu</t>
-        </is>
-      </c>
-      <c r="H10" s="29" t="inlineStr">
-        <is>
-          <t>tak</t>
+          <t>sponsor akademii</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="inlineStr">
+        <is>
+          <t>nie</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="17">
       <c r="A11" s="26" t="inlineStr">
         <is>
-          <t>Nagrania studyjne dziesiątki finalistów</t>
+          <t>Plebiscyt na piosenkę: nabór, ocena, nagrody, prowadzenie</t>
         </is>
       </c>
       <c r="B11" s="26" t="inlineStr">
         <is>
-          <t>możliwość realizacji nagrania studyjnego dla każdego z dziesięciu finalistów; liczba nagrań zależy od przyjęcia oferty, prawa przy autorach</t>
+          <t>plebiscyt i jego laureaci</t>
         </is>
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>2028</t>
+          <t>2027-2028</t>
         </is>
       </c>
       <c r="D11" s="25" t="n">
-        <v>75000</v>
-      </c>
-      <c r="E11" s="28" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>107600</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>28080</v>
       </c>
       <c r="F11" s="25" t="n">
-        <v>75000</v>
+        <v>79520</v>
       </c>
       <c r="G11" s="26" t="inlineStr">
         <is>
@@ -819,29 +819,29 @@
     <row r="12" ht="15" customHeight="1" s="17">
       <c r="A12" s="26" t="inlineStr">
         <is>
-          <t>Hymn z teledyskiem</t>
+          <t>Nagrania studyjne dziesiątki finalistów</t>
         </is>
       </c>
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>nagranie i premiera w czasie trwania naboru</t>
+          <t>możliwość realizacji nagrania studyjnego dla każdego z dziesięciu finalistów; liczba nagrań zależy od przyjęcia oferty, prawa przy autorach</t>
         </is>
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>2028</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>80000</v>
-      </c>
-      <c r="E12" s="25" t="n">
-        <v>80000</v>
-      </c>
-      <c r="F12" s="28" t="inlineStr">
+        <v>75000</v>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>-</t>
         </is>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>75000</v>
       </c>
       <c r="G12" s="26" t="inlineStr">
         <is>
@@ -857,32 +857,28 @@
     <row r="13" ht="15" customHeight="1" s="17">
       <c r="A13" s="26" t="inlineStr">
         <is>
-          <t>Realizacja części artystycznej gali</t>
+          <t>Hymn z teledyskiem</t>
         </is>
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>koncert finałowy</t>
+          <t>nagranie i premiera w czasie trwania naboru</t>
         </is>
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="D13" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
-      </c>
-      <c r="E13" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
-      </c>
-      <c r="F13" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>80000</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>80000</v>
+      </c>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G13" s="26" t="inlineStr">
@@ -899,31 +895,37 @@
     <row r="14" ht="23.25" customHeight="1" s="17">
       <c r="A14" s="26" t="inlineStr">
         <is>
-          <t>Plebiscyt na plakat: nabór, ocena, nagrody, oryginały</t>
+          <t>Realizacja części artystycznej gali</t>
         </is>
       </c>
       <c r="B14" s="26" t="inlineStr">
         <is>
-          <t>plebiscyt, okładka antologii, Archiwum reprodukcji</t>
+          <t>koncert finałowy</t>
         </is>
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>2027-2028</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="n">
-        <v>157552</v>
-      </c>
-      <c r="E14" s="25" t="n">
-        <v>17248</v>
-      </c>
-      <c r="F14" s="25" t="n">
-        <v>140304</v>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
+      </c>
+      <c r="E14" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
+      </c>
+      <c r="F14" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
       </c>
       <c r="G14" s="26" t="inlineStr">
         <is>
-          <t>mecenas plebiscytu na plakat o sztucznej inteligencji</t>
+          <t>sponsor plebiscytu</t>
         </is>
       </c>
       <c r="H14" s="29" t="inlineStr">
@@ -935,33 +937,27 @@
     <row r="15" ht="23.25" customHeight="1" s="17">
       <c r="A15" s="26" t="inlineStr">
         <is>
-          <t>Wystawa przy gali</t>
+          <t>Plebiscyt na plakat: nabór, ocena, nagrody, oryginały</t>
         </is>
       </c>
       <c r="B15" s="26" t="inlineStr">
         <is>
-          <t>dziesięć prac finałowych pokazanych publicznie</t>
+          <t>plebiscyt, okładka antologii, Archiwum reprodukcji</t>
         </is>
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="D15" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
-      </c>
-      <c r="E15" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
-      </c>
-      <c r="F15" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
+          <t>2027-2028</t>
+        </is>
+      </c>
+      <c r="D15" s="25" t="n">
+        <v>157552</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>17248</v>
+      </c>
+      <c r="F15" s="25" t="n">
+        <v>140304</v>
       </c>
       <c r="G15" s="26" t="inlineStr">
         <is>
@@ -977,12 +973,12 @@
     <row r="16" ht="23.25" customHeight="1" s="17">
       <c r="A16" s="26" t="inlineStr">
         <is>
-          <t>Wystawa w galerii sztuki z cichą licytacją, otwierana wernisażem</t>
+          <t>Wystawa przy gali</t>
         </is>
       </c>
       <c r="B16" s="26" t="inlineStr">
         <is>
-          <t>te same prace pokazane po gali, jeżeli galeria zostanie pozyskana</t>
+          <t>dziesięć prac finałowych pokazanych publicznie</t>
         </is>
       </c>
       <c r="C16" s="27" t="inlineStr">
@@ -990,94 +986,94 @@
           <t>2028</t>
         </is>
       </c>
-      <c r="D16" s="32" t="n">
-        <v>4928</v>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
       </c>
       <c r="E16" s="31" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F16" s="31" t="n">
-        <v>4928</v>
+          <t>do wyceny</t>
+        </is>
+      </c>
+      <c r="F16" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
       </c>
       <c r="G16" s="26" t="inlineStr">
         <is>
-          <t>partner galerii</t>
-        </is>
-      </c>
-      <c r="H16" s="27" t="inlineStr">
-        <is>
-          <t>nie</t>
+          <t>mecenas plebiscytu na plakat o sztucznej inteligencji</t>
+        </is>
+      </c>
+      <c r="H16" s="29" t="inlineStr">
+        <is>
+          <t>tak</t>
         </is>
       </c>
     </row>
     <row r="17" ht="23.25" customHeight="1" s="17">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>Plebiscyt na film: nabór, ocena, nagrody, prowadzenie</t>
+          <t>Wystawa w galerii sztuki z cichą licytacją, otwierana wernisażem</t>
         </is>
       </c>
       <c r="B17" s="26" t="inlineStr">
         <is>
-          <t>plebiscyt, dziesięć filmów finałowych, Projektornia i Archiwum</t>
+          <t>te same prace pokazane po gali, jeżeli galeria zostanie pozyskana</t>
         </is>
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>2027-2028</t>
-        </is>
-      </c>
-      <c r="D17" s="25" t="n">
-        <v>264800</v>
-      </c>
-      <c r="E17" s="25" t="n">
-        <v>32032</v>
-      </c>
-      <c r="F17" s="25" t="n">
-        <v>232768</v>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="n">
+        <v>4928</v>
+      </c>
+      <c r="E17" s="31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="31" t="n">
+        <v>4928</v>
       </c>
       <c r="G17" s="26" t="inlineStr">
         <is>
-          <t>sponsor plebiscytu na film o sztucznej inteligencji</t>
-        </is>
-      </c>
-      <c r="H17" s="29" t="inlineStr">
-        <is>
-          <t>tak</t>
+          <t>partner galerii</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="inlineStr">
+        <is>
+          <t>nie</t>
         </is>
       </c>
     </row>
     <row r="18" ht="23.25" customHeight="1" s="17">
       <c r="A18" s="26" t="inlineStr">
         <is>
-          <t>Zwiastuny piątki na gali, a przy pozyskaniu sali także pełne pokazy filmów finałowych</t>
+          <t>Plebiscyt na film: nabór, ocena, nagrody, prowadzenie</t>
         </is>
       </c>
       <c r="B18" s="26" t="inlineStr">
         <is>
-          <t>zwiastuny pięciu filmów na gali, a przy pozyskaniu sali pełne pokazy dziesiątki</t>
+          <t>plebiscyt, dziesięć filmów finałowych, Projektornia i Archiwum</t>
         </is>
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="D18" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
-      </c>
-      <c r="E18" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
-      </c>
-      <c r="F18" s="31" t="inlineStr">
-        <is>
-          <t>do wyceny</t>
-        </is>
+          <t>2027-2028</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>264800</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>32032</v>
+      </c>
+      <c r="F18" s="25" t="n">
+        <v>232768</v>
       </c>
       <c r="G18" s="26" t="inlineStr">
         <is>
@@ -1093,113 +1089,158 @@
     <row r="19" ht="15" customHeight="1" s="17">
       <c r="A19" s="26" t="inlineStr">
         <is>
+          <t>Zwiastuny piątki na gali, a przy pozyskaniu sali także pełne pokazy filmów finałowych</t>
+        </is>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
+        <is>
+          <t>zwiastuny pięciu filmów na gali, a przy pozyskaniu sali pełne pokazy dziesiątki</t>
+        </is>
+      </c>
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
+      </c>
+      <c r="E19" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
+      </c>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>do wyceny</t>
+        </is>
+      </c>
+      <c r="G19" s="26" t="inlineStr">
+        <is>
+          <t>sponsor plebiscytu na film o sztucznej inteligencji</t>
+        </is>
+      </c>
+      <c r="H19" s="29" t="inlineStr">
+        <is>
+          <t>tak</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
           <t>Podcast towarzyszący Nagrodzie</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>bezpłatny materiał edukacyjny</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>2027</t>
         </is>
       </c>
-      <c r="D19" s="31" t="inlineStr">
+      <c r="D20" s="31" t="inlineStr">
         <is>
           <t>do wyceny</t>
         </is>
       </c>
-      <c r="E19" s="31" t="inlineStr">
+      <c r="E20" s="31" t="inlineStr">
         <is>
           <t>do wyceny</t>
         </is>
       </c>
-      <c r="F19" s="31" t="inlineStr">
+      <c r="F20" s="31" t="inlineStr">
         <is>
           <t>do wyceny</t>
         </is>
       </c>
-      <c r="G19" s="26" t="inlineStr">
+      <c r="G20" s="26" t="inlineStr">
         <is>
           <t>sponsor Antologii</t>
         </is>
       </c>
-      <c r="H19" s="29" t="inlineStr">
+      <c r="H20" s="29" t="inlineStr">
         <is>
           <t>tak</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="17">
-      <c r="A21" s="33" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="17"/>
+    <row r="22" ht="15" customHeight="1" s="17">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Razem, wiersze objęte prośbą ("tak")</t>
         </is>
       </c>
-      <c r="D21" s="35">
-        <f>SUMIFS(D6:D19,$H$6:$H$19,"tak")</f>
+      <c r="D22" s="35">
+        <f>SUMIFS(D6:D20,$H$6:$H$20,"tak")</f>
         <v/>
       </c>
-      <c r="E21" s="35">
-        <f>SUMIFS(E6:E19,$H$6:$H$19,"tak")</f>
+      <c r="E22" s="35">
+        <f>SUMIFS(E6:E20,$H$6:$H$20,"tak")</f>
         <v/>
       </c>
-      <c r="F21" s="35">
-        <f>SUMIFS(F6:F19,$H$6:$H$19,"tak")</f>
+      <c r="F22" s="35">
+        <f>SUMIFS(F6:F20,$H$6:$H$20,"tak")</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="17">
-      <c r="A22" s="36" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Razem, wszystkie wycenione pozycje</t>
         </is>
       </c>
-      <c r="D22" s="38">
-        <f>SUM(D6:D19)</f>
+      <c r="D23" s="38">
+        <f>SUM(D6:D20)</f>
         <v/>
       </c>
-      <c r="E22" s="38">
-        <f>SUM(E6:E19)</f>
+      <c r="E23" s="38">
+        <f>SUM(E6:E20)</f>
         <v/>
       </c>
-      <c r="F22" s="38">
-        <f>SUM(F6:F19)</f>
+      <c r="F23" s="38">
+        <f>SUM(F6:F20)</f>
         <v/>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="17">
-      <c r="A24" s="39" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="17"/>
+    <row r="25">
+      <c r="A25" s="39" t="inlineStr">
         <is>
           <t>Pozycje opisane jako "do wyceny" nie wchodzą do sum powyżej; ich wycena powstanie przed złożeniem wniosku.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="17">
-      <c r="A26" s="40" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="17"/>
+    <row r="27" ht="15" customHeight="1" s="17">
+      <c r="A27" s="40" t="inlineStr">
         <is>
           <t>Co oznacza kolumna "W zakresie pytania do MKiDN"</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="17">
-      <c r="A27" s="39" t="inlineStr">
-        <is>
-          <t>Pismo nie jest wnioskiem o dotację i nie zawiera prośby o żadną z kwot wymienionych w tabeli.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="17">
       <c r="A28" s="39" t="inlineStr">
         <is>
-          <t>"tak" - pozycja należy do części artystycznej przedsięwzięcia, której dotyczy pytanie o właściwy Program Ministra i o drogę finansowania. Jest to pytanie o tryb, nie o środki.</t>
+          <t>Pismo nie jest wnioskiem o dotację i nie zawiera prośby o żadną z kwot wymienionych w tabeli.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="17">
       <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>"tak" - pozycja należy do części artystycznej przedsięwzięcia, której dotyczy pytanie o właściwy Program Ministra i o drogę finansowania. Jest to pytanie o tryb, nie o środki.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="39" t="inlineStr">
         <is>
           <t>"nie" - pozycja jest poza tym pytaniem i ma być finansowana z innych źródeł. Wymieniam ją, aby było widoczne, że o tę samą pozycję nie zwracam się jednocześnie do dwóch źródeł.</t>
         </is>

</xml_diff>

<commit_message>
Instalowalna wersja mobilna w Budżecie Uruchomienia
Zamiast osobnej aplikacji w sklepach: ta sama strona dodawana do ekranu
telefonu, z działaniem bez sieci, pobieraniem e-booka i audiobooka do
czytania oraz słuchania offline i powiadomieniami o nowych zgłoszeniach.
Jeden kod i jedno utrzymanie zamiast dwóch sklepów, dwóch procesów
wydawniczych i recenzji przy każdej zmianie regulaminu.

120 godzin, 26 400 zł netto. Budżet Uruchomienia rośnie do 198 380 zł
netto, suma wszystkich wycenionych pozycji do 1 793 466,80 zł. Zakres
objęty pytaniem do MKiDN bez zmian. Pismo uzupełniające opisuje teraz
obie zmiany konstrukcyjne.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/attachments/zestawienie-zadania.xlsx
+++ b/attachments/zestawienie-zadania.xlsx
@@ -714,7 +714,7 @@
       </c>
       <c r="B9" s="26" t="inlineStr">
         <is>
-          <t>fundacja w KRS, regulamin po konsultacji prawnej, cztery narzędzia, przebudowana strona</t>
+          <t>fundacja w KRS, regulamin po konsultacji prawnej, cztery narzędzia, instalowalna wersja mobilna, przebudowana strona</t>
         </is>
       </c>
       <c r="C9" s="27" t="inlineStr">
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="D9" s="25" t="n">
-        <v>164060</v>
+        <v>198380</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>164060</v>
+        <v>198380</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Płatność etapami, jawność wykonawcy i usunięcie sprzeczności w ofertach
Trzy rozstrzygnięcia wprowadzone do wszystkich trzech ofert: płatność
transzami wymagalnymi po odbiorze etapu, narzut liczony wyłącznie od
pracy własnej oraz jawna informacja, że prace wykonuje jednoosobowa
działalność Organizatora, z którą fundacja zawiera umowę.

W ofercie założycielskiej dodatkowo: znak towarowy opisany jako
zgłoszenie, a nie gwarantowana rejestracja; data graniczna 31 grudnia
2027 i tryb przekazania majątku, jeżeli nabór nie ruszy; granice
skrapera; rozdzielenie terminów narzędzi; pierwszeństwo przeniesione na
pozostałe role, bo rola założycielska jest jednorazowa; zastrzeżenie o
kosztach utrzymania narzędzi w kolejnych latach.

Kwoty po podziale ról rozprowadzone do noty koncepcyjnej, uzupełnienia
dla MKiDN, planu działań i linków między ofertami.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/attachments/zestawienie-zadania.xlsx
+++ b/attachments/zestawienie-zadania.xlsx
@@ -687,13 +687,13 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>180362</v>
+        <v>162162</v>
       </c>
       <c r="E8" s="25" t="n">
-        <v>37752</v>
+        <v>33942.4</v>
       </c>
       <c r="F8" s="25" t="n">
-        <v>142610</v>
+        <v>128219.6</v>
       </c>
       <c r="G8" s="26" t="inlineStr">
         <is>
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="D9" s="25" t="n">
-        <v>198380</v>
+        <v>183480</v>
       </c>
       <c r="E9" s="25" t="n">
-        <v>198380</v>
+        <v>183480</v>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>

</xml_diff>